<commit_message>
updates order parts xlsx
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_D_Inverter/Rev04/BOM/BOM_UZ_D_Inverter_Variant_V1_Rev04_ordering_overview.xlsx
+++ b/Project Outputs for UZ_D_Inverter/Rev04/BOM/BOM_UZ_D_Inverter_Variant_V1_Rev04_ordering_overview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UltraZohm\uz_d_inverter\Project Outputs for UZ_D_Inverter\Rev04\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1B1835B-1A9B-4429-9388-67D927C7AE27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C73A1A4-D9F6-4FDB-BEEC-B8F642B91A43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{F1393F58-CEFA-4786-B894-415FB3C9050D}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="203">
   <si>
     <t>Comment</t>
   </si>
@@ -636,6 +636,18 @@
   </si>
   <si>
     <t>both C95204</t>
+  </si>
+  <si>
+    <t>4.7 uF</t>
+  </si>
+  <si>
+    <t>C64A, C64B, C64C, C65A, C65B, C65C</t>
+  </si>
+  <si>
+    <t>C3858973</t>
+  </si>
+  <si>
+    <t>C1608JB1V475M080AC</t>
   </si>
 </sst>
 </file>
@@ -736,7 +748,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -752,7 +764,6 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1214,7 +1225,9 @@
       <c r="G6" s="11" t="s">
         <v>194</v>
       </c>
-      <c r="I6" s="13"/>
+      <c r="I6" t="s">
+        <v>196</v>
+      </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
@@ -1469,7 +1482,7 @@
       <c r="E20" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="I20" s="15" t="s">
+      <c r="I20" t="s">
         <v>196</v>
       </c>
     </row>
@@ -1789,7 +1802,9 @@
       <c r="E37" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="I37" s="15"/>
+      <c r="I37" t="s">
+        <v>196</v>
+      </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
@@ -1807,7 +1822,9 @@
       <c r="E38" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="I38" s="15"/>
+      <c r="I38" t="s">
+        <v>196</v>
+      </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
@@ -1952,7 +1969,24 @@
       <c r="I46" s="13"/>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="I47" s="15"/>
+      <c r="A47" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="I47" t="s">
+        <v>196</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>